<commit_message>
deprecate imageJ and geometry code
</commit_message>
<xml_diff>
--- a/evaluation/function_inventory.xlsx
+++ b/evaluation/function_inventory.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="functions" sheetId="1" r:id="R66478c39e2bb4a43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="modules" sheetId="2" r:id="R0c8fb6524a10428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="functions" sheetId="1" r:id="R465f1b2031554b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="modules" sheetId="2" r:id="Ree33554f9f6348df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2601,10 +2601,14 @@
         <x:v>Given 3 sets of coordinates definin...</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F91"/>
-      <x:c r="G91"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>atan2() and unit-vector algebra</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Its slope and quadrant logic gives the wrong internal bisector in a simple right-angle case; no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
@@ -2620,10 +2624,12 @@
         <x:v>Checks many points (dataframe pt wi...</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>not evaluated</x:v>
+        <x:v>temporarily retained</x:v>
       </x:c>
       <x:c r="F92"/>
-      <x:c r="G92"/>
+      <x:c r="G92" t="str">
+        <x:v>Temporarily retained because selectrandomquad3() and ispt.inside() use it. The spelling and coordinate-indexing defects were fixed in commit 3a1ed6c; review it with the random-quadrat code.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
@@ -2639,10 +2645,14 @@
         <x:v>Convert Cartesian coordinates to po...</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F93"/>
-      <x:c r="G93"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>r = sqrt(x^2 + y^2); theta = atan2(y, x)</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Uses one-argument atan and therefore returns the wrong angle across quadrants.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="str">
@@ -2658,10 +2668,14 @@
         <x:v>Calculates points on a...</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F94"/>
-      <x:c r="G94"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>parametric base R, graphics::symbols(), or sf::st_buffer()</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>A plotting helper with inconsistent output lengths for coordinates outside the circle; no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="str">
@@ -2677,10 +2691,14 @@
         <x:v>Draw a rectangle given a matrix or ...</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F95"/>
-      <x:c r="G95"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>graphics::polygon() or graphics::rect()</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>A trivial base-graphics wrapper with no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
@@ -2696,10 +2714,14 @@
         <x:v>Equation for (half) a canonical...</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F96"/>
-      <x:c r="G96"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>x = cx + rx * cos(theta); y = cy + ry * sin(theta)</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>A plotting helper with inconsistent output lengths for coordinates outside the ellipse; no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
@@ -2715,10 +2737,14 @@
         <x:v>Create a dataframe for a full circl...</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F97"/>
-      <x:c r="G97"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>parametric base R, graphics::symbols(), or sf::st_buffer()</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Inherits circle() output-length failures and has no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="str">
@@ -2734,10 +2760,14 @@
         <x:v>Creates a dataframe for a full elli...</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F98"/>
-      <x:c r="G98"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>x = cx + rx * cos(theta); y = cy + ry * sin(theta)</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Inherits ellipse() output-alignment problems and has no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="str">
@@ -2753,10 +2783,14 @@
         <x:v>Determines whether any of the 4 cor...</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F99"/>
-      <x:c r="G99"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>direct coordinate comparisons or sf::st_intersects()</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Its documented meaning and actual overlap test disagree, including zero-area boundary contact; no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="str">
@@ -2772,10 +2806,12 @@
         <x:v>Checks a vector of coordinates x, y...</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>not evaluated</x:v>
+        <x:v>temporarily retained</x:v>
       </x:c>
       <x:c r="F100"/>
-      <x:c r="G100"/>
+      <x:c r="G100" t="str">
+        <x:v>Temporarily retained because complete.plotmap() uses it. Its half-open boundary rule is intentional; review it with the mapping code.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
@@ -2791,10 +2827,14 @@
         <x:v>Finds the points where a straight l...</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F101"/>
-      <x:c r="G101"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>sf::st_intersection()</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Inherits the fragile slope-intercept calculations and can fail for vertical lines; no caller remains outside the removal set.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="str">
@@ -2810,10 +2850,14 @@
         <x:v>Finds the point where 2 lines inter...</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F102"/>
-      <x:c r="G102"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>sf::st_intersection()</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Produces inconsistent results for vertical, parallel, and coincident lines; no caller remains outside the removal set.</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="str">
@@ -2829,10 +2873,14 @@
         <x:v>Check whether a point x,y falls bet...</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F103"/>
-      <x:c r="G103"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>direct coordinate comparisons or sf::st_intersects()</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>Tests a bounding box rather than true segment membership and handles endpoints inconsistently; no caller remains outside the removal set.</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" t="str">
@@ -2848,10 +2896,12 @@
         <x:v>Check a single pt (x and y) against...</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>not evaluated</x:v>
+        <x:v>temporarily retained</x:v>
       </x:c>
       <x:c r="F104"/>
-      <x:c r="G104"/>
+      <x:c r="G104" t="str">
+        <x:v>Temporarily retained because coverage.diag() uses it. Its result-construction defect was fixed in commit 3a1ed6c; review it with the coverage code.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" t="str">
@@ -2867,10 +2917,14 @@
         <x:v>Finds the point where 2 lines inter...</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F105"/>
-      <x:c r="G105"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>sf::st_intersection()</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Calls the undefined line.intersection() and has no caller outside the removal set.</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="str">
@@ -2886,10 +2940,14 @@
         <x:v>Finds the slope and intercept of th...</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F106"/>
-      <x:c r="G106"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>direct vector algebra or sf</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>The slope-intercept representation gives incorrect results for mixed vertical and finite lines; all remaining callers were removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="str">
@@ -2905,10 +2963,12 @@
         <x:v>Distance from a point to a line (so...</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>not evaluated</x:v>
+        <x:v>temporarily retained</x:v>
       </x:c>
       <x:c r="F107"/>
-      <x:c r="G107"/>
+      <x:c r="G107" t="str">
+        <x:v>Temporarily retained because minum.perpdist() uses it, and majoraxisreg() uses minum.perpdist(). Review that regression chain against maintained major-axis implementations such as smatr::ma().</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" t="str">
@@ -2924,10 +2984,14 @@
         <x:v>Finds the slope and intercept of th...</x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F108"/>
-      <x:c r="G108"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>direct vector algebra or sf</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>The slope-intercept representation handles vertical lines poorly; all callers in R/new were removed with this geometry block.</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="str">
@@ -2943,10 +3007,14 @@
         <x:v>Convert polar coordinates to Cartes...</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F109"/>
-      <x:c r="G109"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>x = r * cos(theta); y = r * sin(theta)</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>The inverse calculation is clearer as direct base R and no caller remains.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" t="str">
@@ -2962,10 +3030,14 @@
         <x:v>Returns intercept and slope of a li...</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F110"/>
-      <x:c r="G110"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>point-direction or normal-form line representation</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>Treats coincident points as a vertical line and is unreliable for mixed scalar and tabular inputs; all remaining callers were removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" t="str">
@@ -2981,10 +3053,14 @@
         <x:v>Draw a line segment between two poi...</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F111"/>
-      <x:c r="G111"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>graphics::segments()</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>A trivial wrapper around base graphics with no remaining caller.</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="str">
@@ -3019,10 +3095,14 @@
         <x:v>Distance between two pairs of x-y c...</x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F113"/>
-      <x:c r="G113"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>sqrt((x1 - x2)^2 + (y1 - y2)^2)</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>A trivial Euclidean-distance wrapper with no remaining caller; direct base R is clearer.</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="str">
@@ -3038,10 +3118,14 @@
         <x:v>Distance between two x-y coordinate...</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F114"/>
-      <x:c r="G114"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>sqrt((pts[, 1] - pts[, 3])^2 + (pts[, 2] - pts[, 4])^2)</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>Duplicates a direct Euclidean-distance calculation and fails when a one-row object is simplified to a vector.</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="str">
@@ -3057,10 +3141,14 @@
         <x:v>Distance between two x-y coordinate...</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F115"/>
-      <x:c r="G115"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>sqrt(rowSums((pt1 - pt2)^2))</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>Duplicates a direct Euclidean-distance calculation and fails when supplied coordinate vectors rather than two-column objects.</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="17">
       <x:c r="A116" s="1" t="str">
@@ -3076,10 +3164,14 @@
         <x:v>Distance between a point and a segment</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F116"/>
-      <x:c r="G116"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>sf::st_distance(); sf::st_nearest_points(); spatstat.geom::project2segment()</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>Can return the correct distance with missing nearest-point coordinates. Maintained spatial implementations cover this task.</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="str">
@@ -4571,10 +4663,14 @@
         <x:v>A version of drop which includes as...</x:v>
       </x:c>
       <x:c r="E191" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F191"/>
-      <x:c r="G191"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F191" t="str">
+        <x:v>drop(as.matrix(x))</x:v>
+      </x:c>
+      <x:c r="G191" t="str">
+        <x:v>All calls were replaced by the exact function body and the auxiliary function was removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="192">
       <x:c r="A192" t="str">
@@ -4725,10 +4821,14 @@
         <x:v>A more convenient version of the R ...</x:v>
       </x:c>
       <x:c r="E199" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F199"/>
-      <x:c r="G199"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F199" t="str">
+        <x:v>if(test) a else b</x:v>
+      </x:c>
+      <x:c r="G199" t="str">
+        <x:v>Its three existing length-comparison calls were replaced with max(length(a), length(b)); the auxiliary function was removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="200">
       <x:c r="A200" t="str">
@@ -4801,10 +4901,14 @@
         <x:v>A form of grep returning logical in...</x:v>
       </x:c>
       <x:c r="E203" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F203"/>
-      <x:c r="G203"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F203" t="str">
+        <x:v>grepl(needle, haystack, fixed = TRUE) %in% TRUE</x:v>
+      </x:c>
+      <x:c r="G203" t="str">
+        <x:v>The replacement preserves the original FALSE result for missing patterns or values; the auxiliary function was removed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="204">
       <x:c r="A204" t="str">
@@ -4953,10 +5057,14 @@
         <x:v>A version of paste with sep=''....</x:v>
       </x:c>
       <x:c r="E211" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F211"/>
-      <x:c r="G211"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F211" t="str">
+        <x:v>paste0()</x:v>
+      </x:c>
+      <x:c r="G211" t="str">
+        <x:v>All existing calls were replaced with paste0(); the substitutions are equivalent for their actual argument structures, although paste0() is not a universal replacement for every hypothetical pst() call.</x:v>
+      </x:c>
     </x:row>
     <x:row r="212">
       <x:c r="A212" t="str">
@@ -4979,7 +5087,7 @@
     </x:row>
     <x:row r="213">
       <x:c r="A213" t="str">
-        <x:v>randomRow</x:v>
+        <x:v>randomElement</x:v>
       </x:c>
       <x:c r="B213" t="str">
         <x:v>01_utilities</x:v>
@@ -7750,10 +7858,14 @@
         <x:v>Called from imageJ.to.lxly where fo...</x:v>
       </x:c>
       <x:c r="E348" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F348"/>
-      <x:c r="G348"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F348" t="str">
+        <x:v>georeference.R</x:v>
+      </x:c>
+      <x:c r="G348" t="str">
+        <x:v>The legacy Condit/ImageJ workflow was replaced by point_clicker(), apply_homography_transformation(), and apply_affine_transformation(); see coordinate-recovery.qmd.</x:v>
+      </x:c>
     </x:row>
     <x:row r="349">
       <x:c r="A349" t="str">
@@ -7769,11 +7881,13 @@
         <x:v>Reads quadrat maps created by image...</x:v>
       </x:c>
       <x:c r="E349" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F349"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F349" t="str">
+        <x:v>georeference.R</x:v>
+      </x:c>
       <x:c r="G349" t="str">
-        <x:v>Removed dependency on deprecated and trivial convert.rowcol()</x:v>
+        <x:v>The legacy Condit/ImageJ workflow was replaced by point_clicker(), apply_homography_transformation(), and apply_affine_transformation(); see coordinate-recovery.qmd.</x:v>
       </x:c>
     </x:row>
     <x:row r="350">
@@ -7790,10 +7904,14 @@
         <x:v>Convert map pixels from digitzing p...</x:v>
       </x:c>
       <x:c r="E350" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F350"/>
-      <x:c r="G350"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F350" t="str">
+        <x:v>georeference.R</x:v>
+      </x:c>
+      <x:c r="G350" t="str">
+        <x:v>The legacy Condit/ImageJ workflow was replaced by point_clicker(), apply_homography_transformation(), and apply_affine_transformation(); see coordinate-recovery.qmd.</x:v>
+      </x:c>
     </x:row>
     <x:row r="351">
       <x:c r="A351" t="str">
@@ -7809,10 +7927,14 @@
         <x:v>This function is called by fullplot...</x:v>
       </x:c>
       <x:c r="E351" t="str">
-        <x:v>not evaluated</x:v>
-      </x:c>
-      <x:c r="F351"/>
-      <x:c r="G351"/>
+        <x:v>deprecated</x:v>
+      </x:c>
+      <x:c r="F351" t="str">
+        <x:v>georeference.R</x:v>
+      </x:c>
+      <x:c r="G351" t="str">
+        <x:v>The legacy Condit/ImageJ workflow was replaced by point_clicker(), apply_homography_transformation(), and apply_affine_transformation(); see coordinate-recovery.qmd.</x:v>
+      </x:c>
     </x:row>
     <x:row r="352">
       <x:c r="A352" t="str">

</xml_diff>